<commit_message>
Update release files for V1.1.0.0
</commit_message>
<xml_diff>
--- a/cfg/CFG_EG1615_EG80132_260514.xlsx
+++ b/cfg/CFG_EG1615_EG80132_260514.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\上位机\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\上位机\cfg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C6A059E-0667-4DE3-81D3-ADC3EBE28CBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{581484D5-C823-4A37-B5CF-3304C3145B33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5775" yWindow="4380" windowWidth="28890" windowHeight="15375" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="APP" sheetId="1" r:id="rId1"/>
@@ -166,7 +166,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1327" uniqueCount="581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1327" uniqueCount="582">
   <si>
     <t>0x55</t>
   </si>
@@ -1945,6 +1945,10 @@
   </si>
   <si>
     <t>频率</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u16</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -9772,7 +9776,7 @@
         <v>55</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>23</v>
+        <v>581</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -10995,15 +10999,14 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="A41:A45"/>
-    <mergeCell ref="B36:B40"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="C18:C20"/>
-    <mergeCell ref="B31:B35"/>
-    <mergeCell ref="C31:C35"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="A31:A35"/>
-    <mergeCell ref="B21:B25"/>
+    <mergeCell ref="B12:B17"/>
+    <mergeCell ref="C3:C7"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="A36:A40"/>
+    <mergeCell ref="C36:C40"/>
+    <mergeCell ref="B3:B7"/>
+    <mergeCell ref="C8:C11"/>
+    <mergeCell ref="A8:A11"/>
     <mergeCell ref="A52:A57"/>
     <mergeCell ref="A26:A30"/>
     <mergeCell ref="B26:B30"/>
@@ -11020,14 +11023,15 @@
     <mergeCell ref="C21:C25"/>
     <mergeCell ref="C41:C45"/>
     <mergeCell ref="A21:A25"/>
-    <mergeCell ref="B12:B17"/>
-    <mergeCell ref="C3:C7"/>
-    <mergeCell ref="A3:A7"/>
-    <mergeCell ref="A36:A40"/>
-    <mergeCell ref="C36:C40"/>
-    <mergeCell ref="B3:B7"/>
-    <mergeCell ref="C8:C11"/>
-    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="A41:A45"/>
+    <mergeCell ref="B36:B40"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="B31:B35"/>
+    <mergeCell ref="C31:C35"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="A31:A35"/>
+    <mergeCell ref="B21:B25"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12874,6 +12878,32 @@
     </row>
   </sheetData>
   <mergeCells count="42">
+    <mergeCell ref="C6:C10"/>
+    <mergeCell ref="A11:A14"/>
+    <mergeCell ref="B11:B14"/>
+    <mergeCell ref="C11:C14"/>
+    <mergeCell ref="C37:C40"/>
+    <mergeCell ref="C26:C28"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="C23:C25"/>
+    <mergeCell ref="B23:B25"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="B6:B10"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="B32:B34"/>
+    <mergeCell ref="A44:A46"/>
+    <mergeCell ref="A29:A31"/>
+    <mergeCell ref="C29:C31"/>
+    <mergeCell ref="C32:C34"/>
+    <mergeCell ref="A41:A43"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="A32:A34"/>
+    <mergeCell ref="C41:C43"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="B26:B28"/>
     <mergeCell ref="B47:B51"/>
     <mergeCell ref="C47:C51"/>
     <mergeCell ref="A15:A16"/>
@@ -12890,32 +12920,6 @@
     <mergeCell ref="A20:A22"/>
     <mergeCell ref="C44:C46"/>
     <mergeCell ref="A37:A40"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="B32:B34"/>
-    <mergeCell ref="A44:A46"/>
-    <mergeCell ref="A29:A31"/>
-    <mergeCell ref="C29:C31"/>
-    <mergeCell ref="C32:C34"/>
-    <mergeCell ref="A41:A43"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="A32:A34"/>
-    <mergeCell ref="C41:C43"/>
-    <mergeCell ref="B29:B31"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="B26:B28"/>
-    <mergeCell ref="C6:C10"/>
-    <mergeCell ref="A11:A14"/>
-    <mergeCell ref="B11:B14"/>
-    <mergeCell ref="C11:C14"/>
-    <mergeCell ref="C37:C40"/>
-    <mergeCell ref="C26:C28"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="C23:C25"/>
-    <mergeCell ref="B23:B25"/>
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="B6:B10"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>